<commit_message>
Concerta lógica de Segmentação
</commit_message>
<xml_diff>
--- a/data/processed/piores_rankings/top 5 piores % Engajamento.xlsx
+++ b/data/processed/piores_rankings/top 5 piores % Engajamento.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:H5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -455,6 +455,174 @@
       <c r="H1" t="inlineStr">
         <is>
           <t>Instagram</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Leonardo Silva Prates</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>PDT - BA</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>dep.leoprates@camara.leg.br</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>(61) 3215-5646</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Gabinete 646 - Anexo IV - Câmara dos Deputados</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>05/04/1978</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Salvador - BA</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/leoprates</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Darci Pompeo De Mattos</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>PDT - RS</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>dep.pompeodemattos@camara.leg.br</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>(61) 3215-5704</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Gabinete 704 - Anexo IV - Câmara dos Deputados</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>12/07/1958</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Santo Augusto - RS</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/pompeodemattospdt</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Vinicius Rapozo De Carvalho</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>REPUBLICANOS - SP</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>dep.viniciuscarvalho@camara.leg.br</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>(61) 3215-5356</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Gabinete 356 - Anexo IV - Câmara dos Deputados</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>07/01/1966</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Rio de Janeiro - RJ</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/viniciuscarvalhooficial</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Vitor Lippi</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>PSD - SP</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>dep.vitorlippi@camara.leg.br</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>(61) 3215-5823</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Gabinete 823 - Anexo IV - Câmara dos Deputados</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>18/05/1959</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Sorocaba - SP</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/vitorlippi</t>
         </is>
       </c>
     </row>

</xml_diff>